<commit_message>
chore: remove temporary lock files and update heatmap export spreadsheet
</commit_message>
<xml_diff>
--- a/exports/Wundauflagen_F1_Heatmap_Vergleich.xlsx
+++ b/exports/Wundauflagen_F1_Heatmap_Vergleich.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mertakdemir/Developer/uni/Modell/exports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77910EEE-C802-8245-AE3A-F1A218D37422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E3A3D09-9CC2-1746-BC87-75F24F0DB042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -620,19 +620,19 @@
     <xf numFmtId="0" fontId="6" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3495,8 +3495,8 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" columnSort="1" ref="A1:BI16">
     <sortCondition descending="1" ref="A8:BI8"/>
   </sortState>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="70" fitToWidth="2" fitToHeight="0" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+  <pageMargins left="0.2" right="0" top="0.2" bottom="0.2" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="43" fitToHeight="0" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 

</xml_diff>